<commit_message>
hydro: AT00 and DE00 run-of-river ramps, and ES00's reservoir floor margin
The last part of the hydro update, from runs of difficult hydro years.

- hydropower-compilation.xlsx: maxRampUp and maxRampDown of AT00 rorTurbine
  0.00231 -> 0.00331 and DE00 rorTurbine 0.00295 -> 0.00395, written in the
  helper table as +0.001. The save also re-pointed the workbook's external link
  to ObservedTrends.xlsx from bb-master to bb-dev; nothing reads it.
- changes.inc: ES00's reservoir floor in f02 is 15 % above the realized floor,
  as FR00's has been since cb96c6c; other storage nodes keep 10 %.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src_files/data_files/hydropower-compilation.xlsx
+++ b/src_files/data_files/hydropower-compilation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BB\bb-dev\north_european_model\src_files\data_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63E8FC15-7493-4D49-B15B-252B3F97727A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45AE226E-B748-4DD7-9F41-D8F68740159E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1080" windowWidth="21600" windowHeight="12585" tabRatio="747" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="747" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodedata" sheetId="13" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="83">
   <si>
     <t>AT00</t>
   </si>
@@ -369,6 +369,9 @@
   </si>
   <si>
     <t>minGenPenalty</t>
+  </si>
+  <si>
+    <t>relative</t>
   </si>
 </sst>
 </file>
@@ -483,7 +486,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -529,6 +532,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -583,7 +592,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -660,6 +669,7 @@
     <xf numFmtId="1" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1076,20 +1086,20 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
+      <sheetData sheetId="14" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -2501,10 +2511,8 @@
       <c r="K1" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="L1" s="11" t="inlineStr">
-        <is>
-          <t>relative</t>
-        </is>
+      <c r="L1" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="O1" t="s">
         <v>47</v>
@@ -3343,7 +3351,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
         <v>2</v>
       </c>
@@ -3524,7 +3532,7 @@
       <c r="J30" s="12"/>
       <c r="K30" s="24"/>
       <c r="L30" s="12">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
@@ -3999,11 +4007,11 @@
       </c>
       <c r="I2" s="32">
         <f t="shared" ref="I2:I33" si="3">IF(ROUND(SUMIFS($AA$8:$AA$42, $Y$8:$Y$42,$A2,    $Z$8:$Z$42,$B2), 5)&gt;0, ROUND(SUMIFS($AA$8:$AA$42, $Y$8:$Y$42,$A2,    $Z$8:$Z$42,$B2), 5), "")</f>
-        <v>2.31E-3</v>
+        <v>3.31E-3</v>
       </c>
       <c r="J2" s="32">
         <f>I2</f>
-        <v>2.31E-3</v>
+        <v>3.31E-3</v>
       </c>
       <c r="K2" s="33">
         <f t="shared" ref="K2:K33" si="4">IF(SUMIFS($AF$7:$AF$19,    $AD$7:$AD$19,$A2,     $AE$7:$AE$19,$B2)&gt;0, SUMIFS($AF$7:$AF$19,    $AD$7:$AD$19,$A2,     $AE$7:$AE$19,$B2), "")</f>
@@ -4149,11 +4157,11 @@
       </c>
       <c r="I5" s="32">
         <f t="shared" si="3"/>
-        <v>2.9499999999999999E-3</v>
+        <v>3.9500000000000004E-3</v>
       </c>
       <c r="J5" s="32">
         <f t="shared" si="6"/>
-        <v>2.9499999999999999E-3</v>
+        <v>3.9500000000000004E-3</v>
       </c>
       <c r="K5" s="33">
         <f t="shared" si="4"/>
@@ -4400,8 +4408,9 @@
       <c r="Z8" t="s">
         <v>49</v>
       </c>
-      <c r="AA8">
-        <v>2.31E-3</v>
+      <c r="AA8" s="34">
+        <f>0.00231+0.001</f>
+        <v>3.31E-3</v>
       </c>
       <c r="AB8">
         <v>0.92500000000000004</v>
@@ -5112,8 +5121,9 @@
       <c r="Z16" t="s">
         <v>49</v>
       </c>
-      <c r="AA16">
-        <v>2.9499999999999999E-3</v>
+      <c r="AA16" s="34">
+        <f>0.00295+0.001</f>
+        <v>3.9500000000000004E-3</v>
       </c>
       <c r="AB16">
         <v>0.61399999999999999</v>

</xml_diff>